<commit_message>
Add annotated structure figures and receptor hotspot analysis for GLP-1R review
Six annotated 3D scenes (key residues labelled on 6X18, 6LN2, 3C5T, 5E94, 5VEW,
6X1A, 6ORV, 6XOX), new report section and sheet on shared vs agonist-selective
receptor residues, Fab 3F52 clash and ECD-boundary robustness checks, annotated
6X18 PDB (class in B-factor column), regenerated XLSX/CSV/REPORT.md, scene scripts.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kmf7NmTar9RFvXanAAMXDG
</commit_message>
<xml_diff>
--- a/glp1r_agonist_vs_antagonist/GLP1R_agonist_vs_antagonist.xlsx
+++ b/glp1r_agonist_vs_antagonist/GLP1R_agonist_vs_antagonist.xlsx
@@ -11,25 +11,27 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Сравнение" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Лиганды" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 SAR пептида" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 PDB реестр" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Чек-лист дизайна" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Расчёт - GLP-1 в 6X18" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Расчёт - состояния" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Расчёт - борозда ECD" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Расчёт - неакт. в акт." sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Источники" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3b Остатки рецептора" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 PDB реестр" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Чек-лист дизайна" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Расчёт - GLP-1 в 6X18" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Расчёт - состояния" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Расчёт - борозда ECD" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Расчёт - неакт. в акт." sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Источники" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Сравнение'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Лиганды'!$A$1:$I$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 SAR пептида'!$A$1:$J$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 PDB реестр'!$A$1:$K$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Чек-лист дизайна'!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6 Расчёт - GLP-1 в 6X18'!$A$1:$D$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7 Расчёт - состояния'!$A$1:$N$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'8 Расчёт - борозда ECD'!$A$1:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'9 Расчёт - неакт. в акт.'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10 Источники'!$A$1:$C$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'3b Остатки рецептора'!$A$1:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'4 PDB реестр'!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'5 Чек-лист дизайна'!$A$1:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'6 Расчёт - GLP-1 в 6X18'!$A$1:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'7 Расчёт - состояния'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'8 Расчёт - борозда ECD'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'9 Расчёт - неакт. в акт.'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'10 Источники'!$A$1:$C$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +515,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Листы: 1) Сравнение — матрица агонист/антагонист; 2) Лиганды — ключевые молекулы с числами; 3) SAR пептида — позиции GLP-1 7–36; 4) PDB реестр — все 80 записей RCSB с UniProt P43220; 5) Чек-лист дизайна; 6–9) Расчёты автора; 10) Источники.</t>
+          <t>Листы: 1) Сравнение — матрица агонист/антагонист; 2) Лиганды — ключевые молекулы с числами; 3) SAR пептида — позиции GLP-1 7–36; 3b) Остатки рецептора — общие и агонист-специфичные; 4) PDB реестр — все 80 записей RCSB с UniProt P43220; 5) Чек-лист дизайна; 6–9) Расчёты автора; 10) Источники.</t>
         </is>
       </c>
     </row>
@@ -559,6 +561,207 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Структура / сравнение</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Остатки ECD (UniProt), скрытые &gt; 10 Å²</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Число остатков</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Скрыто, Å²</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Ex4(9–39), 3C5T (ECD)</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>28 30 31 32 35 36 39 67 68 69 88 90 91 118 121 123 127 128</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>688 (на лиганде)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>GLP-1, 3IOL (изолированный ECD)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>29 30 32 35 36 39 67 68 69 88 89 90 91 121 123 128</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>571 (на лиганде)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>GLP-1, 6X18 (полноразмерный)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>29 30 31 32 35 36 39 43 67 68 69 88 90 91 121 123 128 137</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>651 (на лиганде)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Fab 3F52, 5E94 (эпитоп)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>29 30 31 32 33 35 36 39 40 43 68 137 138 141 142 144 145</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>≈ 970 (на ECD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Совпадение: Ex4(9–39) ∩ GLP-1(3IOL)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>14 общих остатков</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Совпадение: GLP-1 (3IOL) ∩ GLP-1 (6X18)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>15 общих остатков</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr"/>
+      <c r="D7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Совпадение: Fab 3F52 ∩ GLP-1 (3IOL)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>29 30 32 35 36 39 68 — 7 из 16 (44%)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Доступность борозды в закрытой форме (6LN2)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>994 Å² в контексте / 1125 Å² на изолированном ECD = 0.88</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Доступность борозды в 6X18 (рецептор без пептида)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>1022 Å² / 1152 Å² = 0.89</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -661,13 +864,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1525,70 +1728,138 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Страница Challenge 3 (Proteinbase)</t>
+          <t>Coopman K et al. 2011, Mol Endocrinol — мутагенез TMD GLP-1R</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>https://proteinbase.com/competitions/anthropic-adaptyv-2026/challenges/glp1r</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr"/>
+          <t>10.1210/me.2011-1160</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>21868452</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Страница выбора дизайнов (Proteinbase)</t>
+          <t>Xiao Q et al. 2000, J Mol Endocrinol — детерминанты связывания GLP-1R</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>https://proteinbase.com/competitions/anthropic-adaptyv-2026/selection</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr"/>
+          <t>10.1677/jme.0.0250321</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>11116211</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Adaptyv: критерии новизны</t>
+          <t>Wootten D et al. 2013, PNAS — полярные TM-остатки и смещённый агонизм</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>https://www.adaptyvbio.com/blog/novelty</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr"/>
+          <t>10.1073/pnas.1221585110</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>23479653</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>InvivoGen: HEK293 CRE-SEAP GLP-1 биотест (для ориентира по формату теста)</t>
+          <t>Mann RJ et al. 2010, Peptides — Cys226–Cys296</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>https://www.invivogen.com/incretin-bioassay-glp-1-reporter-cell-line</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr"/>
+          <t>10.1016/j.peptides.2010.09.015</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>20869417</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
+          <t>Страница Challenge 3 (Proteinbase)</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>https://proteinbase.com/competitions/anthropic-adaptyv-2026/challenges/glp1r</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Страница выбора дизайнов (Proteinbase)</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>https://proteinbase.com/competitions/anthropic-adaptyv-2026/selection</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Adaptyv: критерии новизны</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>https://www.adaptyvbio.com/blog/novelty</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>InvivoGen: HEK293 CRE-SEAP GLP-1 биотест (для ориентира по формату теста)</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>https://www.invivogen.com/incretin-bioassay-glp-1-reporter-cell-line</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
           <t>RCSB PDB (Search API, Data API), UniProt P43220</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
         <is>
           <t>https://www.rcsb.org</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C56"/>
+  <autoFilter ref="A1:C60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2555,7 +2826,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>ECD, хотспот L95 по нумерации препринта</t>
+          <t>ECD, хотспот «Leu95» (в статье; вероятно, нумерация зрелого белка = L118 в UniProt)</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -4406,6 +4677,669 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Остаток (UniProt P43220)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Элемент</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Контакт с GLP-1 в 6X18 (≤4 Å)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Данные мутагенеза / функции</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Класс</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>T29, V30, L32, T35, V36, W39, E68, Y69, Y88, P90, W91, R121, L123, E128</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>ECD, борозда</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>F28, I29, L32, V33, R36, A25, K26 (GLP-1)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Скрытая поверхность ECD совпадает у Ex4(9–39), GLP-1 (изолированный ECD) и GLP-1 в полноразмерном рецепторе: 14–15 общих остатков (наш расчёт)</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Общий (агонист и антагонист)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Runge 2008; Underwood 2010; расчёт</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>W33</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>ECD</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Приматоспецифичный контакт с LY3502970 (орфорглипрон)</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Малые молекулы</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Kawai 2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Y152</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>TM1</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность и GLP-1, и Ex(9–39)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Общий</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011; Zhang 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>R190</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>TM2</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>E9</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность и GLP-1, и Ex(9–39); полярный контакт R190–E9 в центральной сети активации</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Общий</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011; Zhang 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>K197</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>TM2</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность преимущественно GLP-1; падение потенции больше падения аффинности; K197A ↓ связывания</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011; Xiao 2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>D198</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>TM2</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность только GLP-1</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011; Xiao 2000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Q234</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>TM3</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность преимущественно GLP-1</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Y235</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>TM3</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность и GLP-1, и Ex(9–39)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Общий</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>W284</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ECL2 / верх TM4</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность преимущественно GLP-1; падение потенции больше падения аффинности</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>K288</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ECL2 / TM4</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Ala/Leu резко снижают аффинность пептидов с полным N-концом, но не их N-усечённых аналогов</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный (N-конец)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Al-Sabah &amp; Donnelly 2003</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>T298, R299</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ECL2</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>H7 (R299 — H-связь), S14, S17</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Структурный контакт; R299 дотягивается до H7</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Zhang 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>W306</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ECL3 / верх TM5–6</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>H7, G10, T11</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Структурный контакт</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Расчёт по 6X18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>R310</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>TM5</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность только GLP-1; падение потенции больше падения аффинности</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Агонист-специфичный</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>C347</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>ICL3 / TM6</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Ковалентный сайт аллостерического агониста compound 2 на цитоплазматическом конце TM6</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Аллостерический</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Cong 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>H363, E364</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>TM6</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Ala снижает аффинность обоих лигандов; H363A полностью разобщён с cAMP</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Общий; сопряжение</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Coopman 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>R380, L384, L388</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TM7</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>T11, D15 (R380); A8, T11, D15 (L384); E9, F12 (L388)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Структурные контакты N-конца</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Расчёт по 6X18; Zhang 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>L141, L144, Y148</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>верх TM1</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>F12</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Структурный (гидрофобный) контакт</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Расчёт по 6X18</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Q211, H212</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>ECL1</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>W31 (по Zhang 2017)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Контакт C-концевой части пептида с ECL1 — возможная причина частичного агонизма GLP-1(15–36)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Zhang 2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>C226–C296</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>ECL1–ECL2</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Функциональное сопряжение дисульфида рядом с карманом активации</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Структурный</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Mann 2010</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8531,7 +9465,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8874,7 +9808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9397,7 +10331,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10194,205 +11128,4 @@
   <autoFilter ref="A1:N16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Структура / сравнение</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Остатки ECD (UniProt), скрытые &gt; 10 Å²</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Число остатков</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Скрыто, Å²</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Ex4(9–39), 3C5T (ECD)</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>28 30 31 32 35 36 39 67 68 69 88 90 91 118 121 123 127 128</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>688 (на лиганде)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>GLP-1, 3IOL (изолированный ECD)</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>29 30 32 35 36 39 67 68 69 88 89 90 91 121 123 128</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>571 (на лиганде)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>GLP-1, 6X18 (полноразмерный)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>29 30 31 32 35 36 39 43 67 68 69 88 90 91 121 123 128 137</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>651 (на лиганде)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Fab 3F52, 5E94 (эпитоп)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>29 30 31 32 33 35 36 39 40 43 68 137 138 141 142 144 145</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>≈ 970 (на ECD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Совпадение: Ex4(9–39) ∩ GLP-1(3IOL)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>14 общих остатков</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Совпадение: GLP-1 (3IOL) ∩ GLP-1 (6X18)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>15 общих остатков</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Совпадение: Fab 3F52 ∩ GLP-1 (3IOL)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>29 30 32 35 36 39 68 — 7 из 16 (44%)</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Доступность борозды в закрытой форме (6LN2)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>994 Å² в контексте / 1125 Å² на изолированном ECD = 0.88</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Доступность борозды в 6X18 (рецептор без пептида)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>1022 Å² / 1152 Å² = 0.89</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D10"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>